<commit_message>
FR24 nitel (p/np/u/c) Excel formu + calismayi yapan / tarih
templates/fr24-nitel-sablon.xlsx (erp-araclar/fr24_nitel_sablon.py ile uretilir): FR24
gorunumunde; istatistik, kontrol sinirlari, Surec Z, Cpk esdegeri, degerlendirme ve 4
grafik (kontrol karti, kumulatif, oran-n, histogram) canli formul. Kart turu (p/np/u/c)
ve kabul esigi Excel'de degistirilince her sey yeniden hesaplanir. Excel = ERP
(4 kart turunde oran, Cpk esdegeri, kontrol disi sayisi birebir).
Nitel sayfada 'Excel (FR24)' dugmesi, Tarih ve Calismayi yapan alanlari (kayda yazilir).
FR24 nicel formuna 'Calismayi yapan' satiri (N16); Sorumlu = ERP oturumundaki ad soyad.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/fr24-sablon.xlsx
+++ b/templates/fr24-sablon.xlsx
@@ -2390,6 +2390,19 @@
         <v>108</v>
       </c>
       <c r="F16" s="30"/>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>Çalışmayı yapan</t>
+        </is>
+      </c>
+      <c r="K16" s="7"/>
+      <c r="L16" s="7"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="11"/>
+      <c r="O16" s="5"/>
+      <c r="P16" s="5"/>
+      <c r="Q16" s="5"/>
+      <c r="R16" s="5"/>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
@@ -3316,7 +3329,9 @@
       <c r="D74" s="30"/>
     </row>
   </sheetData>
-  <mergeCells count="82">
+  <mergeCells count="84">
+    <mergeCell ref="J16:M16"/>
+    <mergeCell ref="N16:R16"/>
     <mergeCell ref="N41:R41"/>
     <mergeCell ref="J45:R45"/>
     <mergeCell ref="J18:M18"/>

</xml_diff>